<commit_message>
Update holiday master data
Refresh the loc_holiday.xlsx workbook with the latest holiday records and remove the temporary ~$blocklisted_words.xlsx file left behind by Excel.
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/loc_holiday.xlsx
+++ b/mosip_master/xlsx/loc_holiday.xlsx
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2000001</v>
+        <v>3000001</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2000001</v>
+        <v>3000002</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -542,7 +542,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2000001</v>
+        <v>3000003</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2000002</v>
+        <v>3000004</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2000002</v>
+        <v>3000005</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -647,7 +647,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2000002</v>
+        <v>3000006</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -682,7 +682,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2000003</v>
+        <v>3000007</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2000003</v>
+        <v>3000008</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2000003</v>
+        <v>3000009</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2000004</v>
+        <v>3000010</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -822,7 +822,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2000004</v>
+        <v>3000011</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2000004</v>
+        <v>3000012</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -892,7 +892,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2000005</v>
+        <v>3000013</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2000005</v>
+        <v>3000014</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2000005</v>
+        <v>3000015</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2000006</v>
+        <v>3000016</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2000006</v>
+        <v>3000017</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1067,7 +1067,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2000006</v>
+        <v>3000018</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2000007</v>
+        <v>3000019</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2000007</v>
+        <v>3000020</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2000007</v>
+        <v>3000021</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2000008</v>
+        <v>3000022</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1242,7 +1242,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2000008</v>
+        <v>3000023</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1277,7 +1277,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2000008</v>
+        <v>3000024</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2000009</v>
+        <v>3000025</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2000009</v>
+        <v>3000026</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1382,7 +1382,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2000009</v>
+        <v>3000027</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2000010</v>
+        <v>3000028</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2000010</v>
+        <v>3000029</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2000010</v>
+        <v>3000030</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1522,7 +1522,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2000011</v>
+        <v>3000031</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2000011</v>
+        <v>3000032</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2000011</v>
+        <v>3000033</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2000012</v>
+        <v>3000034</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2000012</v>
+        <v>3000035</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1697,7 +1697,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2000012</v>
+        <v>3000036</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1732,7 +1732,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>2000013</v>
+        <v>3000037</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>2000013</v>
+        <v>3000038</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1802,7 +1802,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2000013</v>
+        <v>3000039</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>2000014</v>
+        <v>3000040</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1872,7 +1872,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2000014</v>
+        <v>3000041</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2000014</v>
+        <v>3000042</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2000015</v>
+        <v>3000043</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2000015</v>
+        <v>3000044</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>2000015</v>
+        <v>3000045</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -2047,7 +2047,7 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2000016</v>
+        <v>3000046</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -2082,7 +2082,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>2000016</v>
+        <v>3000047</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2000016</v>
+        <v>3000048</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>2000017</v>
+        <v>3000049</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2000017</v>
+        <v>3000050</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -2222,7 +2222,7 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>2000017</v>
+        <v>3000051</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -2257,7 +2257,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>2000018</v>
+        <v>3000052</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>2000018</v>
+        <v>3000053</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>2000018</v>
+        <v>3000054</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>2000019</v>
+        <v>3000055</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -2397,7 +2397,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>2000019</v>
+        <v>3000056</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2000019</v>
+        <v>3000057</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>2000020</v>
+        <v>3000058</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -2502,7 +2502,7 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>2000020</v>
+        <v>3000059</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -2537,7 +2537,7 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>2000020</v>
+        <v>3000060</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -2572,7 +2572,7 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>2000021</v>
+        <v>3000061</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>2000021</v>
+        <v>3000062</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -2642,7 +2642,7 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>2000021</v>
+        <v>3000063</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -2677,7 +2677,7 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>2000022</v>
+        <v>3000064</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>2000022</v>
+        <v>3000065</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>2000022</v>
+        <v>3000066</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -2782,7 +2782,7 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>2000023</v>
+        <v>3000067</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>2000023</v>
+        <v>3000068</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -2852,7 +2852,7 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>2000023</v>
+        <v>3000069</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2887,7 +2887,7 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>2000024</v>
+        <v>3000070</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2922,7 +2922,7 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>2000024</v>
+        <v>3000071</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2957,7 +2957,7 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>2000024</v>
+        <v>3000072</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2992,7 +2992,7 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>2000025</v>
+        <v>3000073</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -3027,7 +3027,7 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>2000025</v>
+        <v>3000074</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -3062,7 +3062,7 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>2000025</v>
+        <v>3000075</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>2000026</v>
+        <v>3000076</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>2000026</v>
+        <v>3000077</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -3167,7 +3167,7 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>2000026</v>
+        <v>3000078</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -3202,7 +3202,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>2000027</v>
+        <v>3000079</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>2000027</v>
+        <v>3000080</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -3272,7 +3272,7 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>2000027</v>
+        <v>3000081</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>2000028</v>
+        <v>3000082</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>2000028</v>
+        <v>3000083</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>2000028</v>
+        <v>3000084</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>2000029</v>
+        <v>3000085</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>2000029</v>
+        <v>3000086</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -3482,7 +3482,7 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>2000029</v>
+        <v>3000087</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -3517,7 +3517,7 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>2000030</v>
+        <v>3000088</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -3552,7 +3552,7 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>2000030</v>
+        <v>3000089</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>2000030</v>
+        <v>3000090</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -3622,7 +3622,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>2000031</v>
+        <v>3000091</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -3657,7 +3657,7 @@
         </is>
       </c>
       <c r="B93" t="n">
-        <v>2000031</v>
+        <v>3000092</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -3692,7 +3692,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>2000031</v>
+        <v>3000093</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>2000032</v>
+        <v>3000094</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -3762,7 +3762,7 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>2000032</v>
+        <v>3000095</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>2000032</v>
+        <v>3000096</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -3832,7 +3832,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>2000033</v>
+        <v>3000097</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -3867,7 +3867,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>2000033</v>
+        <v>3000098</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -3902,7 +3902,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>2000033</v>
+        <v>3000099</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>2000034</v>
+        <v>3000100</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -3972,7 +3972,7 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>2000034</v>
+        <v>3000101</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -4007,7 +4007,7 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>2000034</v>
+        <v>3000102</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
@@ -4042,7 +4042,7 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>2000035</v>
+        <v>3000103</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
@@ -4077,7 +4077,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>2000035</v>
+        <v>3000104</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>2000035</v>
+        <v>3000105</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>2000036</v>
+        <v>3000106</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
@@ -4182,7 +4182,7 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>2000036</v>
+        <v>3000107</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>2000036</v>
+        <v>3000108</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
@@ -4252,7 +4252,7 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>2000037</v>
+        <v>3000109</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>2000037</v>
+        <v>3000110</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -4322,7 +4322,7 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>2000037</v>
+        <v>3000111</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
@@ -4357,7 +4357,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>2000038</v>
+        <v>3000112</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -4392,7 +4392,7 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>2000038</v>
+        <v>3000113</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
@@ -4427,7 +4427,7 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>2000038</v>
+        <v>3000114</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>2000039</v>
+        <v>3000115</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
@@ -4497,7 +4497,7 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>2000039</v>
+        <v>3000116</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
@@ -4532,7 +4532,7 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>2000039</v>
+        <v>3000117</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="B119" t="n">
-        <v>2000040</v>
+        <v>3000118</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
@@ -4602,7 +4602,7 @@
         </is>
       </c>
       <c r="B120" t="n">
-        <v>2000040</v>
+        <v>3000119</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>2000040</v>
+        <v>3000120</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>2000041</v>
+        <v>3000121</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>2000041</v>
+        <v>3000122</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -4742,7 +4742,7 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>2000041</v>
+        <v>3000123</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="B125" t="n">
-        <v>2000042</v>
+        <v>3000124</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="B126" t="n">
-        <v>2000042</v>
+        <v>3000125</v>
       </c>
       <c r="C126" t="inlineStr">
         <is>
@@ -4847,7 +4847,7 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>2000042</v>
+        <v>3000126</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -4882,7 +4882,7 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>2000043</v>
+        <v>3000127</v>
       </c>
       <c r="C128" t="inlineStr">
         <is>
@@ -4917,7 +4917,7 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>2000043</v>
+        <v>3000128</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
@@ -4952,7 +4952,7 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>2000043</v>
+        <v>3000129</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="B131" t="n">
-        <v>2000044</v>
+        <v>3000130</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
@@ -5022,7 +5022,7 @@
         </is>
       </c>
       <c r="B132" t="n">
-        <v>2000044</v>
+        <v>3000131</v>
       </c>
       <c r="C132" t="inlineStr">
         <is>
@@ -5057,7 +5057,7 @@
         </is>
       </c>
       <c r="B133" t="n">
-        <v>2000044</v>
+        <v>3000132</v>
       </c>
       <c r="C133" t="inlineStr">
         <is>
@@ -5092,7 +5092,7 @@
         </is>
       </c>
       <c r="B134" t="n">
-        <v>2000045</v>
+        <v>3000133</v>
       </c>
       <c r="C134" t="inlineStr">
         <is>
@@ -5127,7 +5127,7 @@
         </is>
       </c>
       <c r="B135" t="n">
-        <v>2000045</v>
+        <v>3000134</v>
       </c>
       <c r="C135" t="inlineStr">
         <is>
@@ -5162,7 +5162,7 @@
         </is>
       </c>
       <c r="B136" t="n">
-        <v>2000045</v>
+        <v>3000135</v>
       </c>
       <c r="C136" t="inlineStr">
         <is>
@@ -5197,7 +5197,7 @@
         </is>
       </c>
       <c r="B137" t="n">
-        <v>2000046</v>
+        <v>3000136</v>
       </c>
       <c r="C137" t="inlineStr">
         <is>
@@ -5232,7 +5232,7 @@
         </is>
       </c>
       <c r="B138" t="n">
-        <v>2000046</v>
+        <v>3000137</v>
       </c>
       <c r="C138" t="inlineStr">
         <is>
@@ -5267,7 +5267,7 @@
         </is>
       </c>
       <c r="B139" t="n">
-        <v>2000046</v>
+        <v>3000138</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -5302,7 +5302,7 @@
         </is>
       </c>
       <c r="B140" t="n">
-        <v>2000047</v>
+        <v>3000139</v>
       </c>
       <c r="C140" t="inlineStr">
         <is>
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="B141" t="n">
-        <v>2000047</v>
+        <v>3000140</v>
       </c>
       <c r="C141" t="inlineStr">
         <is>
@@ -5372,7 +5372,7 @@
         </is>
       </c>
       <c r="B142" t="n">
-        <v>2000047</v>
+        <v>3000141</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
         </is>
       </c>
       <c r="B143" t="n">
-        <v>2000048</v>
+        <v>3000142</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
@@ -5442,7 +5442,7 @@
         </is>
       </c>
       <c r="B144" t="n">
-        <v>2000048</v>
+        <v>3000143</v>
       </c>
       <c r="C144" t="inlineStr">
         <is>
@@ -5477,7 +5477,7 @@
         </is>
       </c>
       <c r="B145" t="n">
-        <v>2000048</v>
+        <v>3000144</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="B146" t="n">
-        <v>2000049</v>
+        <v>3000145</v>
       </c>
       <c r="C146" t="inlineStr">
         <is>
@@ -5547,7 +5547,7 @@
         </is>
       </c>
       <c r="B147" t="n">
-        <v>2000049</v>
+        <v>3000146</v>
       </c>
       <c r="C147" t="inlineStr">
         <is>
@@ -5582,7 +5582,7 @@
         </is>
       </c>
       <c r="B148" t="n">
-        <v>2000049</v>
+        <v>3000147</v>
       </c>
       <c r="C148" t="inlineStr">
         <is>
@@ -5617,7 +5617,7 @@
         </is>
       </c>
       <c r="B149" t="n">
-        <v>2000050</v>
+        <v>3000148</v>
       </c>
       <c r="C149" t="inlineStr">
         <is>
@@ -5652,7 +5652,7 @@
         </is>
       </c>
       <c r="B150" t="n">
-        <v>2000050</v>
+        <v>3000149</v>
       </c>
       <c r="C150" t="inlineStr">
         <is>
@@ -5687,7 +5687,7 @@
         </is>
       </c>
       <c r="B151" t="n">
-        <v>2000050</v>
+        <v>3000150</v>
       </c>
       <c r="C151" t="inlineStr">
         <is>
@@ -5722,7 +5722,7 @@
         </is>
       </c>
       <c r="B152" t="n">
-        <v>2000051</v>
+        <v>3000151</v>
       </c>
       <c r="C152" t="inlineStr">
         <is>
@@ -5757,7 +5757,7 @@
         </is>
       </c>
       <c r="B153" t="n">
-        <v>2000051</v>
+        <v>3000152</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>
@@ -5792,7 +5792,7 @@
         </is>
       </c>
       <c r="B154" t="n">
-        <v>2000051</v>
+        <v>3000153</v>
       </c>
       <c r="C154" t="inlineStr">
         <is>

</xml_diff>